<commit_message>
✅ Regenerate expected Excel files with is_income column
</commit_message>
<xml_diff>
--- a/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
+++ b/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,6 +531,11 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>is_income</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>category</t>
         </is>
       </c>
@@ -574,7 +579,10 @@
       <c r="J2" t="b">
         <v>0</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>FOOD</t>
         </is>
@@ -591,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,25 +630,30 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>is_income</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>participant</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>original_share</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>original_currency</t>
         </is>
@@ -669,23 +682,26 @@
       <c r="F2" t="b">
         <v>0</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>Alice</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>15</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>15</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>

</xml_diff>

<commit_message>
✅ Regenerate expected Excel files with transaction_ledger sheet
</commit_message>
<xml_diff>
--- a/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
+++ b/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
@@ -12,6 +12,7 @@
     <sheet name="allocations" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="attachments" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="balances" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="transaction_ledger" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -788,4 +789,91 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Alice</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Receipt</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FOOD</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
🐛 Show ledger cost as positive amount and keep dates as datetimes
</commit_message>
<xml_diff>
--- a/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
+++ b/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
@@ -841,10 +841,8 @@
       <c r="A2" t="n">
         <v>0</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2025-01-01</t>
-        </is>
+      <c r="B2" s="1" t="n">
+        <v>45658.5</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -862,7 +860,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-15</v>
+        <v>15</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Transaction Ledger Sheet (split view sheet) (#73)
* ✨ Add transaction_ledger sheet with per-member net position per entry

* ✅ Regenerate expected Excel files with transaction_ledger sheet

* 🎨 Format transaction ledger code

* 🐛 Show ledger cost as positive amount and keep dates as datetimes

---------

Co-authored-by: kemal.erbakirci <kemal.erbakirci@adevinta.com>
Co-authored-by: wenceslas-sanchez <wenceslas.sanchez@msci.com>
</commit_message>
<xml_diff>
--- a/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
+++ b/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
@@ -12,6 +12,7 @@
     <sheet name="allocations" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="attachments" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="balances" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="transaction_ledger" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -788,4 +789,89 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Alice</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>45658.5</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Receipt</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FOOD</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>